<commit_message>
Updated GBSC with Brazil data
</commit_message>
<xml_diff>
--- a/InputData/elec/GBSC/Grid Battery Storage Capacities.xlsx
+++ b/InputData/elec/GBSC/Grid Battery Storage Capacities.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shigu\Documents\_swj\_Talanoa\CPSA Fletcher\dados\InputData (BR) 2024\d08 elec\GBSC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saido\OneDrive\Documents\eps-brazil-cpl\InputData\elec\GBSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD5D175E-4F07-4504-B816-EF0365057661}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1536" yWindow="1536" windowWidth="18912" windowHeight="9900" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1530" yWindow="1530" windowWidth="18915" windowHeight="9900" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -24,7 +23,7 @@
   <definedNames>
     <definedName name="gigwatts_to_megawatts">About!#REF!</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -528,7 +527,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="_([$€-2]* #,##0.00_);_([$€-2]* \(#,##0.00\);_([$€-2]* &quot;-&quot;??_)"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
@@ -1099,71 +1098,71 @@
     </xf>
   </cellXfs>
   <cellStyles count="65">
-    <cellStyle name="20% - Accent1 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
-    <cellStyle name="20% - Accent2 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
-    <cellStyle name="20% - Accent3 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
-    <cellStyle name="20% - Accent4 2" xfId="5" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
-    <cellStyle name="20% - Accent5 2" xfId="6" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
-    <cellStyle name="20% - Accent6 2" xfId="7" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
-    <cellStyle name="40% - Accent1 2" xfId="8" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="40% - Accent2 2" xfId="9" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
-    <cellStyle name="40% - Accent3 2" xfId="10" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
-    <cellStyle name="40% - Accent4 2" xfId="11" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
-    <cellStyle name="40% - Accent5 2" xfId="12" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
-    <cellStyle name="40% - Accent6 2" xfId="13" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
-    <cellStyle name="60% - Accent1 2" xfId="14" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
-    <cellStyle name="60% - Accent2 2" xfId="15" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
-    <cellStyle name="60% - Accent3 2" xfId="16" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
-    <cellStyle name="60% - Accent4 2" xfId="17" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
-    <cellStyle name="60% - Accent5 2" xfId="18" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
-    <cellStyle name="60% - Accent6 2" xfId="19" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
-    <cellStyle name="Accent1 2" xfId="20" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
-    <cellStyle name="Accent2 2" xfId="21" xr:uid="{00000000-0005-0000-0000-000013000000}"/>
-    <cellStyle name="Accent3 2" xfId="22" xr:uid="{00000000-0005-0000-0000-000014000000}"/>
-    <cellStyle name="Accent4 2" xfId="23" xr:uid="{00000000-0005-0000-0000-000015000000}"/>
-    <cellStyle name="Accent5 2" xfId="24" xr:uid="{00000000-0005-0000-0000-000016000000}"/>
-    <cellStyle name="Accent6 2" xfId="25" xr:uid="{00000000-0005-0000-0000-000017000000}"/>
-    <cellStyle name="Bad 2" xfId="26" xr:uid="{00000000-0005-0000-0000-000018000000}"/>
-    <cellStyle name="Body: normal cell" xfId="55" xr:uid="{00000000-0005-0000-0000-000019000000}"/>
-    <cellStyle name="Body: normal cell 2" xfId="62" xr:uid="{C847FCFE-E55D-4040-9145-A5096CF2655C}"/>
-    <cellStyle name="Calculation 2" xfId="27" xr:uid="{00000000-0005-0000-0000-00001A000000}"/>
-    <cellStyle name="Check Cell 2" xfId="28" xr:uid="{00000000-0005-0000-0000-00001B000000}"/>
-    <cellStyle name="Euro" xfId="29" xr:uid="{00000000-0005-0000-0000-00001C000000}"/>
-    <cellStyle name="Explanatory Text 2" xfId="30" xr:uid="{00000000-0005-0000-0000-00001D000000}"/>
-    <cellStyle name="Font: Calibri, 9pt regular" xfId="51" xr:uid="{00000000-0005-0000-0000-00001E000000}"/>
-    <cellStyle name="Font: Calibri, 9pt regular 2" xfId="58" xr:uid="{78094820-C238-4C9A-89E8-C7624DC87CE5}"/>
-    <cellStyle name="Footnotes: top row" xfId="56" xr:uid="{00000000-0005-0000-0000-00001F000000}"/>
-    <cellStyle name="Footnotes: top row 2" xfId="63" xr:uid="{09E8E243-1470-4CD0-B658-C11350CB5319}"/>
-    <cellStyle name="Good 2" xfId="31" xr:uid="{00000000-0005-0000-0000-000020000000}"/>
-    <cellStyle name="Header: bottom row" xfId="52" xr:uid="{00000000-0005-0000-0000-000021000000}"/>
-    <cellStyle name="Header: bottom row 2" xfId="59" xr:uid="{A013B94F-3E32-4EB8-A68D-C3E5ECFDA1D8}"/>
-    <cellStyle name="Heading 1 2" xfId="32" xr:uid="{00000000-0005-0000-0000-000022000000}"/>
-    <cellStyle name="Heading 2 2" xfId="33" xr:uid="{00000000-0005-0000-0000-000023000000}"/>
-    <cellStyle name="Heading 3 2" xfId="34" xr:uid="{00000000-0005-0000-0000-000024000000}"/>
-    <cellStyle name="Heading 4 2" xfId="35" xr:uid="{00000000-0005-0000-0000-000025000000}"/>
-    <cellStyle name="Hiperlink" xfId="64" builtinId="8"/>
-    <cellStyle name="Input 2" xfId="36" xr:uid="{00000000-0005-0000-0000-000027000000}"/>
-    <cellStyle name="Linked Cell 2" xfId="37" xr:uid="{00000000-0005-0000-0000-000028000000}"/>
-    <cellStyle name="Neutral 2" xfId="38" xr:uid="{00000000-0005-0000-0000-000029000000}"/>
+    <cellStyle name="20% - Accent1 2" xfId="2"/>
+    <cellStyle name="20% - Accent2 2" xfId="3"/>
+    <cellStyle name="20% - Accent3 2" xfId="4"/>
+    <cellStyle name="20% - Accent4 2" xfId="5"/>
+    <cellStyle name="20% - Accent5 2" xfId="6"/>
+    <cellStyle name="20% - Accent6 2" xfId="7"/>
+    <cellStyle name="40% - Accent1 2" xfId="8"/>
+    <cellStyle name="40% - Accent2 2" xfId="9"/>
+    <cellStyle name="40% - Accent3 2" xfId="10"/>
+    <cellStyle name="40% - Accent4 2" xfId="11"/>
+    <cellStyle name="40% - Accent5 2" xfId="12"/>
+    <cellStyle name="40% - Accent6 2" xfId="13"/>
+    <cellStyle name="60% - Accent1 2" xfId="14"/>
+    <cellStyle name="60% - Accent2 2" xfId="15"/>
+    <cellStyle name="60% - Accent3 2" xfId="16"/>
+    <cellStyle name="60% - Accent4 2" xfId="17"/>
+    <cellStyle name="60% - Accent5 2" xfId="18"/>
+    <cellStyle name="60% - Accent6 2" xfId="19"/>
+    <cellStyle name="Accent1 2" xfId="20"/>
+    <cellStyle name="Accent2 2" xfId="21"/>
+    <cellStyle name="Accent3 2" xfId="22"/>
+    <cellStyle name="Accent4 2" xfId="23"/>
+    <cellStyle name="Accent5 2" xfId="24"/>
+    <cellStyle name="Accent6 2" xfId="25"/>
+    <cellStyle name="Bad 2" xfId="26"/>
+    <cellStyle name="Body: normal cell" xfId="55"/>
+    <cellStyle name="Body: normal cell 2" xfId="62"/>
+    <cellStyle name="Calculation 2" xfId="27"/>
+    <cellStyle name="Check Cell 2" xfId="28"/>
+    <cellStyle name="Euro" xfId="29"/>
+    <cellStyle name="Explanatory Text 2" xfId="30"/>
+    <cellStyle name="Font: Calibri, 9pt regular" xfId="51"/>
+    <cellStyle name="Font: Calibri, 9pt regular 2" xfId="58"/>
+    <cellStyle name="Footnotes: top row" xfId="56"/>
+    <cellStyle name="Footnotes: top row 2" xfId="63"/>
+    <cellStyle name="Good 2" xfId="31"/>
+    <cellStyle name="Header: bottom row" xfId="52"/>
+    <cellStyle name="Header: bottom row 2" xfId="59"/>
+    <cellStyle name="Heading 1 2" xfId="32"/>
+    <cellStyle name="Heading 2 2" xfId="33"/>
+    <cellStyle name="Heading 3 2" xfId="34"/>
+    <cellStyle name="Heading 4 2" xfId="35"/>
+    <cellStyle name="Input 2" xfId="36"/>
+    <cellStyle name="Lien hypertexte" xfId="64" builtinId="8"/>
+    <cellStyle name="Linked Cell 2" xfId="37"/>
+    <cellStyle name="Neutral 2" xfId="38"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-00002B000000}"/>
-    <cellStyle name="Normal 2 2" xfId="44" xr:uid="{00000000-0005-0000-0000-00002C000000}"/>
-    <cellStyle name="Normal 2 3" xfId="47" xr:uid="{00000000-0005-0000-0000-00002D000000}"/>
-    <cellStyle name="Normal 2 4" xfId="48" xr:uid="{00000000-0005-0000-0000-00002E000000}"/>
-    <cellStyle name="Normal 2 5" xfId="49" xr:uid="{00000000-0005-0000-0000-00002F000000}"/>
-    <cellStyle name="Normal 2 6" xfId="50" xr:uid="{00000000-0005-0000-0000-000030000000}"/>
-    <cellStyle name="Normal 3" xfId="45" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
-    <cellStyle name="Normal 4" xfId="46" xr:uid="{00000000-0005-0000-0000-000032000000}"/>
-    <cellStyle name="Normal 5" xfId="57" xr:uid="{BB67FBA3-26D7-431F-A684-0CCDA93EC42D}"/>
-    <cellStyle name="Note 2" xfId="39" xr:uid="{00000000-0005-0000-0000-000033000000}"/>
-    <cellStyle name="Output 2" xfId="40" xr:uid="{00000000-0005-0000-0000-000034000000}"/>
-    <cellStyle name="Parent row" xfId="54" xr:uid="{00000000-0005-0000-0000-000035000000}"/>
-    <cellStyle name="Parent row 2" xfId="61" xr:uid="{DAA11FF9-1C05-45C6-8502-434090995867}"/>
-    <cellStyle name="Table title" xfId="53" xr:uid="{00000000-0005-0000-0000-000036000000}"/>
-    <cellStyle name="Table title 2" xfId="60" xr:uid="{D91F8C64-535F-417E-A952-541EE8F2C1E7}"/>
-    <cellStyle name="Title 2" xfId="41" xr:uid="{00000000-0005-0000-0000-000037000000}"/>
-    <cellStyle name="Total 2" xfId="42" xr:uid="{00000000-0005-0000-0000-000038000000}"/>
-    <cellStyle name="Warning Text 2" xfId="43" xr:uid="{00000000-0005-0000-0000-000039000000}"/>
+    <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Normal 2 2" xfId="44"/>
+    <cellStyle name="Normal 2 3" xfId="47"/>
+    <cellStyle name="Normal 2 4" xfId="48"/>
+    <cellStyle name="Normal 2 5" xfId="49"/>
+    <cellStyle name="Normal 2 6" xfId="50"/>
+    <cellStyle name="Normal 3" xfId="45"/>
+    <cellStyle name="Normal 4" xfId="46"/>
+    <cellStyle name="Normal 5" xfId="57"/>
+    <cellStyle name="Note 2" xfId="39"/>
+    <cellStyle name="Output 2" xfId="40"/>
+    <cellStyle name="Parent row" xfId="54"/>
+    <cellStyle name="Parent row 2" xfId="61"/>
+    <cellStyle name="Table title" xfId="53"/>
+    <cellStyle name="Table title 2" xfId="60"/>
+    <cellStyle name="Title 2" xfId="41"/>
+    <cellStyle name="Total 2" xfId="42"/>
+    <cellStyle name="Warning Text 2" xfId="43"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1179,9 +1178,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1219,9 +1218,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1256,7 +1255,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1291,7 +1290,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1464,121 +1463,121 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B22"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.88671875" customWidth="1"/>
-    <col min="2" max="2" width="60.6640625" customWidth="1"/>
+    <col min="1" max="1" width="17.85546875" customWidth="1"/>
+    <col min="2" max="2" width="60.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" s="2"/>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B5" s="2"/>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="22" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="23" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>155</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A9" r:id="rId1" xr:uid="{20F86130-4D79-4501-B792-ABE3E5276337}"/>
+    <hyperlink ref="A9" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId2"/>
@@ -1586,16 +1585,16 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AK114"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="32.109375" customWidth="1"/>
-    <col min="2" max="2" width="45.6640625" customWidth="1"/>
+    <col min="1" max="1" width="32.140625" customWidth="1"/>
+    <col min="2" max="2" width="45.7109375" customWidth="1"/>
     <col min="38" max="38" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B1" s="8" t="s">
         <v>125</v>
       </c>
@@ -1702,8 +1701,8 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:37" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:37" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C3" s="4" t="s">
         <v>1</v>
       </c>
@@ -1714,7 +1713,7 @@
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
     </row>
-    <row r="4" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C4" s="4" t="s">
         <v>2</v>
       </c>
@@ -1727,7 +1726,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C5" s="4" t="s">
         <v>4</v>
       </c>
@@ -1738,7 +1737,7 @@
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
     </row>
-    <row r="6" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C6" s="4" t="s">
         <v>5</v>
       </c>
@@ -1749,7 +1748,7 @@
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
     </row>
-    <row r="10" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>6</v>
       </c>
@@ -1757,12 +1756,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="8" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="8" t="s">
         <v>9</v>
       </c>
@@ -1872,7 +1871,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="13" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="9" t="s">
         <v>10</v>
       </c>
@@ -1982,18 +1981,18 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="14" spans="1:37" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="15" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:37" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="11" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>13</v>
       </c>
@@ -2106,7 +2105,7 @@
         <v>-1.4527999999999999E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>15</v>
       </c>
@@ -2219,7 +2218,7 @@
         <v>-1.2109E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>17</v>
       </c>
@@ -2332,7 +2331,7 @@
         <v>2.2502999999999999E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>19</v>
       </c>
@@ -2445,7 +2444,7 @@
         <v>8.456E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>21</v>
       </c>
@@ -2558,7 +2557,7 @@
         <v>-5.6340000000000001E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>23</v>
       </c>
@@ -2671,7 +2670,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:37" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:37" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="17" t="s">
         <v>25</v>
       </c>
@@ -2784,7 +2783,7 @@
         <v>0.123014</v>
       </c>
     </row>
-    <row r="24" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>27</v>
       </c>
@@ -2897,7 +2896,7 @@
         <v>5.8900000000000003E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>29</v>
       </c>
@@ -3010,7 +3009,7 @@
         <v>2.3185000000000001E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>31</v>
       </c>
@@ -3123,7 +3122,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="27" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>34</v>
       </c>
@@ -3236,12 +3235,12 @@
         <v>1.1344E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="11" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="29" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>37</v>
       </c>
@@ -3354,7 +3353,7 @@
         <v>-3.3660000000000001E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>39</v>
       </c>
@@ -3467,7 +3466,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>41</v>
       </c>
@@ -3580,7 +3579,7 @@
         <v>-9.9999999999999995E-7</v>
       </c>
     </row>
-    <row r="32" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>42</v>
       </c>
@@ -3693,7 +3692,7 @@
         <v>-9.68E-4</v>
       </c>
     </row>
-    <row r="33" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
         <v>43</v>
       </c>
@@ -3806,7 +3805,7 @@
         <v>6.6000000000000005E-5</v>
       </c>
     </row>
-    <row r="34" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>44</v>
       </c>
@@ -3919,12 +3918,12 @@
         <v>-4.06E-4</v>
       </c>
     </row>
-    <row r="36" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="11" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="37" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
         <v>46</v>
       </c>
@@ -4037,7 +4036,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="38" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
         <v>47</v>
       </c>
@@ -4150,7 +4149,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="39" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
         <v>48</v>
       </c>
@@ -4263,7 +4262,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="40" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
         <v>49</v>
       </c>
@@ -4376,7 +4375,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="41" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
         <v>50</v>
       </c>
@@ -4489,7 +4488,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="42" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
         <v>52</v>
       </c>
@@ -4602,7 +4601,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="43" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
         <v>53</v>
       </c>
@@ -4715,7 +4714,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="44" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
         <v>54</v>
       </c>
@@ -4828,7 +4827,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="45" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
         <v>55</v>
       </c>
@@ -4941,7 +4940,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="46" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
         <v>56</v>
       </c>
@@ -5054,7 +5053,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="47" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
         <v>58</v>
       </c>
@@ -5167,12 +5166,12 @@
         <v>33</v>
       </c>
     </row>
-    <row r="48" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="11" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="49" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
         <v>60</v>
       </c>
@@ -5285,7 +5284,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="50" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
         <v>61</v>
       </c>
@@ -5398,7 +5397,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="51" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
         <v>62</v>
       </c>
@@ -5511,7 +5510,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="52" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
         <v>63</v>
       </c>
@@ -5624,7 +5623,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="53" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
         <v>64</v>
       </c>
@@ -5737,7 +5736,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="54" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
         <v>65</v>
       </c>
@@ -5850,7 +5849,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="55" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
         <v>66</v>
       </c>
@@ -5963,7 +5962,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="56" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
         <v>67</v>
       </c>
@@ -6076,7 +6075,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="57" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
         <v>68</v>
       </c>
@@ -6189,7 +6188,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="58" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
         <v>69</v>
       </c>
@@ -6302,7 +6301,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="59" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
         <v>70</v>
       </c>
@@ -6415,7 +6414,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="60" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
         <v>71</v>
       </c>
@@ -6528,12 +6527,12 @@
         <v>33</v>
       </c>
     </row>
-    <row r="62" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B62" s="11" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="63" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
         <v>73</v>
       </c>
@@ -6646,7 +6645,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="64" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
         <v>74</v>
       </c>
@@ -6759,7 +6758,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="65" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
         <v>75</v>
       </c>
@@ -6872,7 +6871,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="66" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
         <v>76</v>
       </c>
@@ -6985,7 +6984,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="67" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
         <v>77</v>
       </c>
@@ -7098,7 +7097,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="68" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
         <v>78</v>
       </c>
@@ -7211,7 +7210,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="69" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
         <v>79</v>
       </c>
@@ -7324,7 +7323,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="70" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
         <v>80</v>
       </c>
@@ -7437,7 +7436,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="71" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
         <v>81</v>
       </c>
@@ -7550,7 +7549,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="72" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
         <v>82</v>
       </c>
@@ -7663,7 +7662,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="74" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="5" t="s">
         <v>83</v>
       </c>
@@ -7776,12 +7775,12 @@
         <v>1.1053E-2</v>
       </c>
     </row>
-    <row r="76" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B76" s="11" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="77" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="5" t="s">
         <v>86</v>
       </c>
@@ -7894,7 +7893,7 @@
         <v>-9.3640000000000008E-3</v>
       </c>
     </row>
-    <row r="78" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="5" t="s">
         <v>87</v>
       </c>
@@ -8007,7 +8006,7 @@
         <v>-2.039E-3</v>
       </c>
     </row>
-    <row r="79" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="5" t="s">
         <v>89</v>
       </c>
@@ -8120,7 +8119,7 @@
         <v>2.5253000000000001E-2</v>
       </c>
     </row>
-    <row r="80" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="s">
         <v>91</v>
       </c>
@@ -8233,7 +8232,7 @@
         <v>-7.0799999999999997E-4</v>
       </c>
     </row>
-    <row r="81" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="s">
         <v>93</v>
       </c>
@@ -8346,7 +8345,7 @@
         <v>6.0502E-2</v>
       </c>
     </row>
-    <row r="82" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="5" t="s">
         <v>94</v>
       </c>
@@ -8459,7 +8458,7 @@
         <v>4.0169999999999997E-3</v>
       </c>
     </row>
-    <row r="83" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="s">
         <v>96</v>
       </c>
@@ -8572,7 +8571,7 @@
         <v>4.7788999999999998E-2</v>
       </c>
     </row>
-    <row r="85" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="5" t="s">
         <v>97</v>
       </c>
@@ -8685,8 +8684,8 @@
         <v>33</v>
       </c>
     </row>
-    <row r="86" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="87" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="87" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B87" s="25" t="s">
         <v>99</v>
       </c>
@@ -8726,137 +8725,137 @@
       <c r="AJ87" s="25"/>
       <c r="AK87" s="25"/>
     </row>
-    <row r="88" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B88" s="6" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="89" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B89" s="6" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="90" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B90" s="6" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="91" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B91" s="6" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="92" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B92" s="6" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="93" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B93" s="6" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="94" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B94" s="6" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="95" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B95" s="6" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="96" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B96" s="6" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="97" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B97" s="6" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="98" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B98" s="6" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="99" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B99" s="6" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="100" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B100" s="6" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="101" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B101" s="6" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="102" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B102" s="6" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="103" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B103" s="6" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="104" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B104" s="6" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="105" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B105" s="6" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="106" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B106" s="6" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="107" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B107" s="6" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="108" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B108" s="6" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="109" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B109" s="6" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="110" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B110" s="6" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="111" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B111" s="6" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="112" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B112" s="6" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="113" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B113" s="6" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="114" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B114" s="6" t="s">
         <v>140</v>
       </c>
@@ -8870,14 +8869,14 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9057A661-82DA-40AC-BC4D-86F55C2ECF27}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AH2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.33203125" customWidth="1"/>
+    <col min="1" max="1" width="19.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>156</v>
       </c>
@@ -8981,7 +8980,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>157</v>
       </c>
@@ -9091,14 +9090,14 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81C0DF4B-0F33-4735-AA0B-51508EB4510E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AH2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>156</v>
       </c>
@@ -9202,7 +9201,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:34" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:34" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="24" t="s">
         <v>158</v>
       </c>
@@ -9312,17 +9311,17 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AF3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33.109375" customWidth="1"/>
+    <col min="1" max="1" width="33.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>120</v>
       </c>
@@ -9420,7 +9419,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>122</v>
       </c>
@@ -9437,114 +9436,115 @@
         <v>0</v>
       </c>
       <c r="F2" s="3">
-        <f>(F1-$E1)/7*$L$2</f>
-        <v>2428.5714285714284</v>
+        <f>E2</f>
+        <v>0</v>
       </c>
       <c r="G2" s="3">
-        <f t="shared" ref="G2:K2" si="0">(G1-$E1)/7*$L$2</f>
-        <v>4857.1428571428569</v>
+        <f t="shared" ref="G2:AF2" si="0">F2</f>
+        <v>0</v>
       </c>
       <c r="H2" s="3">
         <f t="shared" si="0"/>
-        <v>7285.7142857142853</v>
+        <v>0</v>
       </c>
       <c r="I2" s="3">
         <f t="shared" si="0"/>
-        <v>9714.2857142857138</v>
+        <v>0</v>
       </c>
       <c r="J2" s="3">
         <f t="shared" si="0"/>
-        <v>12142.857142857143</v>
+        <v>0</v>
       </c>
       <c r="K2" s="3">
         <f t="shared" si="0"/>
-        <v>14571.428571428571</v>
+        <v>0</v>
       </c>
       <c r="L2" s="3">
-        <v>17000</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="M2" s="3">
-        <f>$L$2*'DRC-BDRC'!O2/'DRC-BDRC'!$N$2</f>
-        <v>17544</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="N2" s="3">
-        <f>$L$2*'DRC-BDRC'!P2/'DRC-BDRC'!$N$2</f>
-        <v>18105.407999999996</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="O2" s="3">
-        <f>$L$2*'DRC-BDRC'!Q2/'DRC-BDRC'!$N$2</f>
-        <v>18414.294904898696</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="P2" s="3">
-        <f>$L$2*'DRC-BDRC'!R2/'DRC-BDRC'!$N$2</f>
-        <v>18714.628443069516</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="Q2" s="3">
-        <f>$L$2*'DRC-BDRC'!S2/'DRC-BDRC'!$N$2</f>
-        <v>19015.789726407547</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="R2" s="3">
-        <f>$L$2*'DRC-BDRC'!T2/'DRC-BDRC'!$N$2</f>
-        <v>19314.605731771804</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="S2" s="3">
-        <f>$L$2*'DRC-BDRC'!U2/'DRC-BDRC'!$N$2</f>
-        <v>19603.212880073756</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="T2" s="3">
-        <f>$L$2*'DRC-BDRC'!V2/'DRC-BDRC'!$N$2</f>
-        <v>19896.924456906861</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="U2" s="3">
-        <f>$L$2*'DRC-BDRC'!W2/'DRC-BDRC'!$N$2</f>
-        <v>20170.494234671096</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="V2" s="3">
-        <f>$L$2*'DRC-BDRC'!X2/'DRC-BDRC'!$N$2</f>
-        <v>20448.340695799267</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="W2" s="3">
-        <f>$L$2*'DRC-BDRC'!Y2/'DRC-BDRC'!$N$2</f>
-        <v>20713.357106835618</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="X2" s="3">
-        <f>$L$2*'DRC-BDRC'!Z2/'DRC-BDRC'!$N$2</f>
-        <v>20986.926884599849</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="Y2" s="3">
-        <f>$L$2*'DRC-BDRC'!AA2/'DRC-BDRC'!$N$2</f>
-        <v>21258.841172029646</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="Z2" s="3">
-        <f>$L$2*'DRC-BDRC'!AB2/'DRC-BDRC'!$N$2</f>
-        <v>21536.825590685687</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="AA2" s="3">
-        <f>$L$2*'DRC-BDRC'!AC2/'DRC-BDRC'!$N$2</f>
-        <v>21797.1514457745</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="AB2" s="3">
-        <f>$L$2*'DRC-BDRC'!AD2/'DRC-BDRC'!$N$2</f>
-        <v>22017.331660253425</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="AC2" s="3">
-        <f>$L$2*'DRC-BDRC'!AE2/'DRC-BDRC'!$N$2</f>
-        <v>22245.513411348755</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="AD2" s="3">
-        <f>$L$2*'DRC-BDRC'!AF2/'DRC-BDRC'!$N$2</f>
-        <v>22464.314050548994</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="AE2" s="3">
-        <f>$L$2*'DRC-BDRC'!AG2/'DRC-BDRC'!$N$2</f>
-        <v>22692.081929060711</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="AF2" s="3">
-        <f>$L$2*'DRC-BDRC'!AH2/'DRC-BDRC'!$N$2</f>
-        <v>22909.778908038003</v>
-      </c>
-    </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
@@ -9560,18 +9560,18 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AF2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="47.109375" customWidth="1"/>
-    <col min="2" max="32" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="47.140625" customWidth="1"/>
+    <col min="2" max="32" width="10.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>120</v>
       </c>
@@ -9669,7 +9669,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>121</v>
       </c>
@@ -9804,18 +9804,18 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.44140625" customWidth="1"/>
-    <col min="2" max="2" width="12.44140625" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>120</v>
       </c>
@@ -9823,7 +9823,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>124</v>
       </c>
@@ -9831,7 +9831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B3" s="3"/>
     </row>
   </sheetData>

</xml_diff>